<commit_message>
Add new Excel files for Monopunto and Multipunto data
- Created new Excel file: "5150 Datos Monopunto CCPP AMANIEL Y LIMON.xlsx"
- Created new Excel file: "7667 Datos Monopunto CCPP AMANIEL Y LIMON.xlsx"
- Created new Excel file: "7455 Datos Multipunto CCPP ORFILIA 5.xlsx"
</commit_message>
<xml_diff>
--- a/MONOPUNTO/1775 Datos Monopunto SERGANO, S.A.xlsx
+++ b/MONOPUNTO/1775 Datos Monopunto SERGANO, S.A.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N11"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -426,11 +426,11 @@
     <col width="21" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
     <col width="8" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
@@ -1009,6 +1009,106 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>NEXUS</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>46212</v>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>46568</v>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>46213</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>0.215785</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.183585</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.14633</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0.121653</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0.105064</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0.125185</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>NEXUS</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>46212</v>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>46568</v>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>46213</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="M13" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>